<commit_message>
REL-012: la M.02 e il caso corretto del collaudo T1 rigenerati con la 1.6.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FwSMQGQ3E2CtzqcjNTREF3
</commit_message>
<xml_diff>
--- a/docs/collaudi/REL-012/fase-2/distinta/distinta.xlsx
+++ b/docs/collaudi/REL-012/fase-2/distinta/distinta.xlsx
@@ -598,7 +598,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Allegata alla tavola M.02, rev. 00 del 2026-10-29. Regole della distinta cfc42a99c0fd0a1a. Quantità indicative.</t>
+          <t>Committente: Committente (dati omessi). Indirizzo: Indirizzo omesso. Allegata alla tavola M.02, rev. 00 del 29.10.2026. Regole della distinta dea73506dac30790. Quantità indicative.</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Si compilano solo le celle gialle, in € oltre IVA: prezzo unitario e importo per le sezioni B-F e H, importo a corpo per la sezione G, solo prezzo unitario per le varianti V (fuori dal totale). Righe grigie: fornite da Nove C o del Committente, non si quotano. Le righe DA DEFINIRE aspettano un dato del progettista.</t>
+          <t>Si compilano solo le celle gialle, in € oltre IVA: prezzo unitario e importo per le sezioni B-F e H, importo a corpo per la sezione G, solo prezzo unitario per le varianti V (fuori dal totale). Righe grigie: forniture escluse da questa offerta (vedi la colonna Fornitura), non si quotano. Le righe DA DEFINIRE aspettano un dato del progettista.</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>A. Apparecchiature (fornite da Nove C, posa dell'installatore)</t>
+          <t>A. Apparecchiature (posa dell'installatore; chi le fornisce: colonna Fornitura)</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>scarico</t>
+          <t>AL-01</t>
         </is>
       </c>
       <c r="G44" s="11" t="n"/>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>sifone</t>
+          <t>SIF-01</t>
         </is>
       </c>
       <c r="G45" s="11" t="n"/>
@@ -2247,7 +2247,7 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>F. Assistenze murarie (aperture comprese; chiusure e ripristini del Committente)</t>
+          <t>F. Assistenze murarie (aperture comprese)</t>
         </is>
       </c>
       <c r="B61" s="6" t="n"/>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>scarico</t>
+          <t>AL-01</t>
         </is>
       </c>
       <c r="G67" s="11" t="n"/>
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="D72" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>Aeff min.: B1 0,05 m², B2 0,052 m², B3 0,039 m², B4 0,051 m², B5 0,051 m²</t>
+          <t>Aeff min.: Camera 13 m² 0,05 m², Camera 15 m² 0,052 m², Camera 16 m² 0,039 m², Soggiorno-cucina 0,102 m²</t>
         </is>
       </c>
       <c r="G72" s="9" t="n"/>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>UI-01 - sifone - scarico</t>
+          <t>UI-01 - SIF-01 - AL-01</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -4252,7 +4252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4330,7 +4330,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §2, proposta 5 approvata dal PO («flessibili ≤ 3 m/s»); proposta 3 (flessibili Ø200 a 2,4-2,6 m/s)</t>
+          <t>regola Nove C per il comfort acustico (mandata fino a 3 m/s)</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4362,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §2, proposta 5 approvata dal PO («flessibili ≤ 3 m/s»); proposta 3 (flessibili Ø200 a 2,4-2,6 m/s)</t>
+          <t>regola Nove C per il comfort acustico (mandata fino a 3 m/s)</t>
         </is>
       </c>
     </row>
@@ -4394,7 +4394,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §2, proposta 5 approvata dal PO («flessibili ≤ 3 m/s»); proposta 3 (flessibili Ø200 a 2,4-2,6 m/s)</t>
+          <t>regola Nove C per il comfort acustico (mandata fino a 3 m/s)</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §2, proposta 5 approvata dal PO («flessibili ≤ 3 m/s»); proposta 3 (flessibili Ø200 a 2,4-2,6 m/s)</t>
+          <t>regola Nove C per il comfort acustico (mandata fino a 3 m/s)</t>
         </is>
       </c>
     </row>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §2, proposta 5 approvata dal PO («flessibili ≤ 3 m/s»); proposta 3 (flessibili Ø200 a 2,4-2,6 m/s)</t>
+          <t>regola Nove C per il comfort acustico (mandata fino a 3 m/s)</t>
         </is>
       </c>
     </row>
@@ -4490,14 +4490,14 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §2, proposta 5 («ripresa &lt; 2 m/s»), sulla sezione lorda; REVISIONE-INDIPENDENTE.md rilievo 4 (1,9 m/s lordi diventano ~3 m/s reali con griglia e filtro)</t>
+          <t>regola Nove C per il comfort acustico (ripresa fino a 2 m/s)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>Camera 13 m²</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -4522,14 +4522,14 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 («griglie di transito a 1,5 m/s»)</t>
+          <t>regola Nove C per il ritorno dell'aria (1,5 m/s nelle griglie di transito)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>Camera 15 m²</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -4554,14 +4554,14 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 («griglie di transito a 1,5 m/s»)</t>
+          <t>regola Nove C per il ritorno dell'aria (1,5 m/s nelle griglie di transito)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>Camera 16 m²</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -4586,14 +4586,14 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 («griglie di transito a 1,5 m/s»)</t>
+          <t>regola Nove C per il ritorno dell'aria (1,5 m/s nelle griglie di transito)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>Soggiorno-cucina</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -4603,12 +4603,12 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>275 m³/h a 1,5 m/s</t>
+          <t>550 m³/h a 1,5 m/s</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Aeff ≥ 0,051 m²</t>
+          <t>Aeff ≥ 0,102 m²</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -4618,46 +4618,46 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 («griglie di transito a 1,5 m/s»)</t>
+          <t>regola Nove C per il ritorno dell'aria (1,5 m/s nelle griglie di transito)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>B5</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>griglia di transito</t>
+          <t>lunghezza della linea frigorifera</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>275 m³/h a 1,5 m/s</t>
+          <t>12 m da quotare</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Aeff ≥ 0,051 m²</t>
+          <t>≤ 30 m (UE-01)</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>da rispettare</t>
+          <t>entro</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 («griglie di transito a 1,5 m/s»)</t>
+          <t>scheda tecnica dell'unità esterna (lunghezza massima della linea)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -4682,29 +4682,29 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 (massimo 30 m dalla scheda Daikin RXM-A, citata in RAPPORTO.md §10)</t>
+          <t>scheda tecnica dell'unità esterna (lunghezza massima della linea)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>T08</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>lunghezza della linea frigorifera</t>
+          <t>scritta sulla tavola</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>12 m da quotare</t>
+          <t>«Ø200 · 270 m³/h · L 6 m»</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>≤ 30 m (UE-01)</t>
+          <t>L 6 m da quotare</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -4714,14 +4714,14 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 (massimo 30 m dalla scheda Daikin RXM-A, citata in RAPPORTO.md §10)</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -4731,12 +4731,12 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>«Ø200 · 270 m³/h · L 6 m»</t>
+          <t>«Ø200 · 280 m³/h · L 3,5 m»</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>L 6 m da quotare</t>
+          <t>L 3,5 m da quotare</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -4746,14 +4746,14 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -4763,12 +4763,12 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>«Ø200 · 280 m³/h · L 3,5 m»</t>
+          <t>«Ø200 · 210 m³/h · L 6 m»</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>L 3,5 m da quotare</t>
+          <t>L 6 m da quotare</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
@@ -4778,14 +4778,14 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -4795,12 +4795,12 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>«Ø200 · 210 m³/h · L 6 m»</t>
+          <t>«Ø200 · 275 m³/h · L 3,5 m»</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>L 6 m da quotare</t>
+          <t>L 3,5 m da quotare</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -4810,14 +4810,14 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -4827,12 +4827,12 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>«Ø200 · 275 m³/h · L 3,5 m»</t>
+          <t>«Ø200 · 275 m³/h · L 7 m»</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>L 3,5 m da quotare</t>
+          <t>L 7 m da quotare</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -4842,14 +4842,14 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -4859,12 +4859,12 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>«Ø200 · 275 m³/h · L 7 m»</t>
+          <t>«Ø6,35 (1/4") · L 12 m»</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>L 7 m da quotare</t>
+          <t>L 12 m da quotare</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -4874,14 +4874,14 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>«Ø6,35 (1/4") · L 12 m»</t>
+          <t>«Ø12,7 (1/2") · L 12 m»</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -4906,14 +4906,14 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>T08</t>
+          <t>T09</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -4923,12 +4923,12 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>«Ø12,7 (1/2") · L 12 m»</t>
+          <t>«PVC Ø32 · L 10 m»</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>L 12 m da quotare</t>
+          <t>L 10 m da quotare</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -4938,14 +4938,14 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>T09</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -4955,12 +4955,12 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>«PVC Ø32 · L 10 m»</t>
+          <t>«3G2,5 · L 20 m»</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>L 10 m da quotare</t>
+          <t>L 20 m da quotare</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -4970,14 +4970,14 @@
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -4987,12 +4987,12 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>«3G2,5 · L 20 m»</t>
+          <t>«3G1,5 · L 15 m»</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>L 20 m da quotare</t>
+          <t>L 15 m da quotare</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -5002,14 +5002,14 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>T11</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -5019,12 +5019,12 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>«3G1,5 · L 15 m»</t>
+          <t>«4G1,5 · L 13 m»</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>L 15 m da quotare</t>
+          <t>L 13 m da quotare</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -5034,14 +5034,14 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -5051,29 +5051,29 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>«4G1,5 · L 13 m»</t>
+          <t>«P1-P2 · L 3 m»</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>L 13 m da quotare</t>
+          <t>L 5 m da quotare</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>entro</t>
+          <t>oltre</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -5083,29 +5083,29 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>«P1-P2 · L 3 m»</t>
+          <t>«P1-P2 · L 5,5 m»</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>L 5 m da quotare</t>
+          <t>L 5,5 m da quotare</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>oltre</t>
+          <t>entro</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -5115,12 +5115,12 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>«P1-P2 · L 5,5 m»</t>
+          <t>«bus · L 9 m»</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>L 5,5 m da quotare</t>
+          <t>L 9 m da quotare</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -5130,14 +5130,14 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -5147,12 +5147,12 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>«bus · L 9 m»</t>
+          <t>«bus · L 7 m»</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>L 9 m da quotare</t>
+          <t>L 7 m da quotare</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -5162,14 +5162,14 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -5179,12 +5179,12 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>«bus · L 7 m»</t>
+          <t>«bus · L 7,5 m»</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>L 7 m da quotare</t>
+          <t>L 7,5 m da quotare</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -5194,14 +5194,14 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T18</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -5211,12 +5211,12 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>«bus · L 7,5 m»</t>
+          <t>«bus · L 5,5 m»</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>L 7,5 m da quotare</t>
+          <t>L 5,5 m da quotare</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -5226,39 +5226,7 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>T18</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>scritta sulla tavola</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>«bus · L 5,5 m»</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>L 5,5 m da quotare</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>entro</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>contratto con REL-012: la scritta di un tratto («Ø200 · L 6 m») è un dato del progettista</t>
+          <t>confronto con la scritta della tratta sulla tavola</t>
         </is>
       </c>
     </row>
@@ -5279,14 +5247,14 @@
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>Da dove viene ogni quantità — la regola, il conto, la fonte, il perché</t>
+          <t>Da dove viene ogni quantità — la voce, il conto, la fonte, il perché</t>
         </is>
       </c>
     </row>
@@ -5298,7 +5266,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Regola</t>
+          <t>Voce</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -5325,17 +5293,17 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>corredo/wired-remote/apparecchiatura</t>
+          <t>Comando a filo dell'unità: Daikin Madoka BRC1H52W</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>1 nel grafo (CF-01)</t>
+          <t>1 nello schema (CF-01)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voci A.5, E.13, F.7</t>
+          <t>regola Nove C per gli apparecchi a parete</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -5352,17 +5320,17 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>corredo/zoning-plenum-5/apparecchiatura</t>
+          <t>Plenum motorizzato di zona a cinque serrande: Airzone Easyzone 5 × Ø200, es. AZEZ8DAIBS07M5 · 1425×250×454 mm</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>1 nel grafo (PLZ-01)</t>
+          <t>1 nello schema (PLZ-01)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voci A.3, B.10, B.11, Z.2</t>
+          <t>regola Nove C per la posa del plenum di zona</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -5379,17 +5347,17 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>corredo/room-thermostat/apparecchiatura</t>
+          <t>Termostato di zona: Airzone Blueface</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>4 nel grafo (TZ-01, TZ-02, TZ-03, TZ-04)</t>
+          <t>4 nello schema (TZ-01, TZ-02, TZ-03, TZ-04)</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voci A.4, E.13, F.7</t>
+          <t>regola Nove C per gli apparecchi a parete</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -5406,17 +5374,17 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>corredo/split-outdoor-unit/apparecchiatura</t>
+          <t>Unità esterna split a pompa di calore: Daikin RXM60A · 49 kg</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>1 nel grafo (UE-01)</t>
+          <t>1 nello schema (UE-01)</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voci A.1, C.5, C.6, C.8, C.9, F.1; REVISIONE-INDIPENDENTE.md rilievo 18</t>
+          <t>regola Nove C per la posa dell'unità esterna</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -5433,17 +5401,17 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>corredo/ducted-indoor-unit/apparecchiatura</t>
+          <t>Unità interna canalizzata ad espansione diretta: Daikin FBA60A9 · 1000×800×245 mm · 35 kg</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>1 nel grafo (UI-01)</t>
+          <t>1 nello schema (UI-01)</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voci A.2, B.4, B.10, D.2, Z.1, Z.2; REVISIONE-INDIPENDENTE.md rilievi 4, 6</t>
+          <t>regola Nove C per la posa dell'unità interna canalizzata</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -5460,7 +5428,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>fluidi/supply_air/flessibile-in-confezioni</t>
+          <t>Condotto flessibile coibentato Ø200 (isolamento 25 mm, barriera vapore), confezione da 10 m</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -5470,7 +5438,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py (confezioni da 10 m, 0,5 m di sfrido, almeno 1,25 × la lunghezza); REVISIONE-INDIPENDENTE.md rilievo 17</t>
+          <t>regola Nove C per i canali flessibili</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -5487,7 +5455,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>fluidi/supply_air/curva-in-lamiera</t>
+          <t>Curva 90° Ø200 in lamiera zincata, all'uscita del plenum</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -5497,7 +5465,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py (4 curve alle uscite con cambio di direzione stretto, scritte a mano sul caso)</t>
+          <t>regola Nove C per i canali flessibili</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -5514,7 +5482,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>fluidi/supply_air/manicotto-di-riserva</t>
+          <t>Manicotto di giunzione Ø200</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -5524,7 +5492,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py («Manicotto di giunzione Ø200», n 2, riserva)</t>
+          <t>regola Nove C per i canali flessibili</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -5541,7 +5509,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>fluidi/supply_air/fascette</t>
+          <t>Fascetta di serraggio Ø200 (anima e mantello)</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -5551,7 +5519,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: REVISIONE-INDIPENDENTE.md rilievo 17 («fascette ≥ 32 con le curve»); lavoro/dimensionamento.py, 36 fascette</t>
+          <t>regola Nove C per i canali flessibili</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -5568,7 +5536,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>fluidi/supply_air/nastro-alluminio</t>
+          <t>Nastro alluminio rinforzato 50 mm</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -5578,7 +5546,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py (2 rotoli per 26 m di flessibile); il passo di 20 m è della sessione di sviluppo, che riproduce il kit: da confermare</t>
+          <t>stima Nove C (un rotolo ogni 20 m di flessibile)</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -5595,7 +5563,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>fluidi/supply_air/sostegni</t>
+          <t>Sostegno per flessibile (fascia o collare con pendino), passo ≤ 1,2 m</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -5605,7 +5573,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 («sostegni ogni ≤ 1,2 m»); lavoro/dimensionamento.py, 25 sostegni</t>
+          <t>regola Nove C per i canali flessibili</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -5622,7 +5590,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>corredo/air-supply-terminal/plenum-porta-bocchetta</t>
+          <t>Plenum porta-bocchetta coibentato per bocchetta 400×200, attacco Ø200 laterale o dall'alto</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -5632,7 +5600,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce B.2; REVISIONE-INDIPENDENTE.md rilievo 5 («il plenum da ordinare sulle bocchette scelte non si può prezzare»)</t>
+          <t>regola Nove C per le bocchette di mandata</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -5649,7 +5617,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>corredo/zoning-plenum-5/kit-sospensione + corredo/return-air-terminal/kit-sospensione + corredo/ducted-indoor-unit/kit-sospensione</t>
+          <t>Kit sospensione: barra filettata M10, tassello per solaio in laterocemento, antivibrante</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -5659,7 +5627,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 («kit sospensione: UI 4, plenum 4, ripresa 2»)</t>
+          <t>regola Nove C per la posa del plenum di zona; regola Nove C per la ripresa dell'aria; regola Nove C per la posa dell'unità interna canalizzata</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -5676,7 +5644,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>corredo/zoning-plenum-5/isolamento-raccordi-plenum</t>
+          <t>Isolamento elastomerico adesivo per raccordi e plenum</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -5686,7 +5654,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce B.11</t>
+          <t>regola Nove C per la posa del plenum di zona</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -5703,7 +5671,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>corredo/return-air-terminal/plenum-di-ripresa</t>
+          <t>Plenum di ripresa coibentato con filtro ispezionabile, bocca 1000×250, sulla bocca di aspirazione dell'unità interna</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -5713,7 +5681,7 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce B.3; REVISIONE-INDIPENDENTE.md rilievo 4 (un solo filtro, nel plenum)</t>
+          <t>regola Nove C per la ripresa dell'aria</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
@@ -5730,7 +5698,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>corredo/ducted-indoor-unit/giunto-antivibrante-ripresa</t>
+          <t>Giunto antivibrante in tela fra unità interna e plenum di ripresa</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -5740,7 +5708,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce B.4</t>
+          <t>regola Nove C per la posa dell'unità interna canalizzata</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -5757,7 +5725,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>fluidi/refrigerant_liquid/tubo-rame-liquido</t>
+          <t>Tubo rame ricotto pre-isolato Ø6,35 (1/4"), isolamento ≥ 10 mm, resistente a 120 °C</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -5767,7 +5735,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 «Refrigerante» (isolamento dal manuale di installazione Daikin FTXM60-71A, citato in RAPPORTO.md §10)</t>
+          <t>manuale di installazione del costruttore della macchina (isolamento delle linee)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -5784,7 +5752,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>fluidi/refrigerant_liquid/manicotti-a-brasare-liquido</t>
+          <t>Manicotto a brasare Ø6,35 (1/4") (riserva, posa in tratta unica)</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -5794,7 +5762,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py («Manicotto a brasare 1/4" e 1/2"», n 4 per le due linee)</t>
+          <t>regola Nove C per le linee frigorifere</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -5811,7 +5779,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>fluidi/refrigerant_gas/tubo-rame-gas</t>
+          <t>Tubo rame ricotto pre-isolato Ø12,7 (1/2"), isolamento ≥ 13 mm, resistente a 120 °C</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -5821,7 +5789,7 @@
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 «Refrigerante» (manuale di installazione Daikin FTXM60-71A, citato in RAPPORTO.md §10)</t>
+          <t>manuale di installazione del costruttore della macchina (isolamento delle linee)</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
@@ -5838,7 +5806,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>fluidi/refrigerant_gas/manicotti-a-brasare-gas</t>
+          <t>Manicotto a brasare Ø12,7 (1/2") (riserva, posa in tratta unica)</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -5848,7 +5816,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py («Manicotto a brasare 1/4" e 1/2"», n 4 per le due linee)</t>
+          <t>regola Nove C per le linee frigorifere</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -5865,7 +5833,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>fluidi/refrigerant_gas/nastro-e-manicotti-isolanti</t>
+          <t>Nastro di finitura e manicotti isolanti per le giunzioni a cartella</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -5875,7 +5843,7 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce C.4</t>
+          <t>regola Nove C per le linee frigorifere</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -5892,7 +5860,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>fluidi/refrigerant_gas/collari-linee-frigo</t>
+          <t>Collare di sostegno linee frigorifere in controsoffitto</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -5902,7 +5870,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce C.7 (10 collari per 12 m)</t>
+          <t>regola Nove C per le linee frigorifere</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -5919,7 +5887,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>fluidi/refrigerant_gas/carica-aggiuntiva</t>
+          <t>Refrigerante R32, riserva per carica aggiuntiva</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -5929,7 +5897,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 (precarica fino a 10 m, oltre 20 g/m: scheda Daikin RXM-A, citata in RAPPORTO.md §10); REVISIONE-INDIPENDENTE.md rilievo 18 (riserva di 0,2 kg)</t>
+          <t>scheda tecnica dell'unità esterna (precarica e carica aggiuntiva)</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -5946,7 +5914,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>corredo/split-outdoor-unit/canalina-esterna</t>
+          <t>Canalina coprilinee esterna 80×60</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
@@ -5956,7 +5924,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce C.5; REVISIONE-INDIPENDENTE.md rilievo 18</t>
+          <t>regola Nove C per la posa dell'unità esterna</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -5973,7 +5941,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>corredo/split-outdoor-unit/accessori-canalina</t>
+          <t>Accessori canalina: curva 2, terminale a muro 1, giunto 2</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -5983,7 +5951,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce C.6; REVISIONE-INDIPENDENTE.md rilievo 18 («canalina con accessori a numero»)</t>
+          <t>regola Nove C per la posa dell'unità esterna</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
@@ -6000,7 +5968,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>corredo/split-outdoor-unit/staffe-unita-esterna</t>
+          <t>Staffe a parete per unità esterna, portata almeno doppia del peso della macchina, con antivibranti</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
@@ -6010,7 +5978,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce C.8 (portata ≥ 100 kg per 49 kg)</t>
+          <t>regola Nove C per la posa dell'unità esterna</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -6027,7 +5995,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>corredo/split-outdoor-unit/scarico-condensa-unita-esterna</t>
+          <t>Scarico condensa dell'unità esterna (funziona anche in caldo): raccordo e tubo Ø16 fino a pluviale o pozzetto</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -6037,7 +6005,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce C.9; REVISIONE-INDIPENDENTE.md rilievo 18</t>
+          <t>regola Nove C per la posa dell'unità esterna</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -6054,7 +6022,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>fluidi/condensate/tubo-pvc</t>
+          <t>Tubo PVC rigido Ø32</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -6064,7 +6032,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 «Condensa»</t>
+          <t>regola Nove C per lo scarico della condensa</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -6081,7 +6049,7 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>fluidi/condensate/curve-condensa</t>
+          <t>Curva 87°-90° Ø32</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -6091,7 +6059,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce D.3 (6 curve su 10 m); il passo è della sessione di sviluppo, che riproduce il kit: da confermare</t>
+          <t>stima Nove C (una curva ogni 2 m)</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -6108,7 +6076,7 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>fluidi/condensate/manicotti-condensa</t>
+          <t>Manicotto Ø32</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -6118,7 +6086,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce D.4 (3 manicotti su 10 m); barre da 3 m, assunzione della sessione di sviluppo: da confermare</t>
+          <t>stima Nove C (barre da 3 m)</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -6135,7 +6103,7 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>fluidi/condensate/collari-condensa</t>
+          <t>Collare per tubo condensa</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -6145,7 +6113,7 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce D.7 (10 collari su 10 m)</t>
+          <t>regola Nove C per lo scarico della condensa</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -6162,7 +6130,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>fluidi/condensate/isolamento-anticondensa</t>
+          <t>Isolamento anticondensa 9 mm per il tubo della condensa</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -6172,7 +6140,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce D.8 (5 m, il solo tratto in controsoffitto, scritto a mano sul caso)</t>
+          <t>regola Nove C per lo scarico della condensa</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -6189,7 +6157,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>fluidi/condensate/collante-pvc</t>
+          <t>Collante e pulitore PVC</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -6199,7 +6167,7 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce D.9</t>
+          <t>regola Nove C per lo scarico della condensa</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -6216,17 +6184,17 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>corredo/condensate-outlet/innesto-sullo-scarico</t>
+          <t>Innesto sullo scarico esistente (braga 45° o presa sul sifone di un apparecchio)</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>scarico: 1</t>
+          <t>AL-01: 1</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce D.6</t>
+          <t>regola Nove C per lo scarico della condensa</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -6243,17 +6211,17 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>corredo/condensate-trap/sifone</t>
+          <t>Sifone ispezionabile per condensa</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>sifone: 1</t>
+          <t>SIF-01: 1</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce D.5</t>
+          <t>regola Nove C per lo scarico della condensa</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -6270,7 +6238,7 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>corredo/ducted-indoor-unit/raccordo-condensa-unita-interna</t>
+          <t>Raccordo di adattamento dall'attacco condensa dell'unità interna (VP20 (Øe 26)) al tubo di scarico, con fascetta</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -6280,7 +6248,7 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce D.2; REVISIONE-INDIPENDENTE.md rilievo 6</t>
+          <t>scheda tecnica dell'unità interna (attacco della condensa)</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -6297,7 +6265,7 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>fluidi/power_supply/cavo-di-alimentazione</t>
+          <t>Cavo FG16OR16 3G2,5, Alimentazione unita' esterna</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -6307,7 +6275,7 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 «Elettrico e bus» (linea dedicata in FG16OR16); la sezione del cavo è un dato del progettista (`sezione` del tratto)</t>
+          <t>regola Nove C per le linee elettriche dedicate</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -6324,7 +6292,7 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>fluidi/power_supply/cavo-di-alimentazione</t>
+          <t>Cavo FG16OR16 3G1,5, Alimentazione centrale Airzone</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
@@ -6334,7 +6302,7 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 «Elettrico e bus» (linea dedicata in FG16OR16); la sezione del cavo è un dato del progettista (`sezione` del tratto)</t>
+          <t>regola Nove C per le linee elettriche dedicate</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -6351,7 +6319,7 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>fluidi/power_supply/protezione-della-linea</t>
+          <t>Magnetotermico-differenziale 1P+N C16, Idn 30 mA, tipo A o F, 6 kA, linea dedicata: Alimentazione unita' esterna</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
@@ -6361,7 +6329,7 @@
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7; REVISIONE-INDIPENDENTE.md rilievi 7 e 12 (la protezione della centrale a sé, verificare la targa della macchina)</t>
+          <t>targa della macchina (dato del progettista)</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -6378,7 +6346,7 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>fluidi/power_supply/protezione-della-linea</t>
+          <t>Magnetotermico 1P+N C6, linea dedicata: Alimentazione centrale Airzone</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
@@ -6388,7 +6356,7 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7; REVISIONE-INDIPENDENTE.md rilievi 7 e 12 (la protezione della centrale a sé, verificare la targa della macchina)</t>
+          <t>targa della macchina (dato del progettista)</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -6405,7 +6373,7 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>fluidi/power_supply/scatola-di-derivazione</t>
+          <t>Scatola di derivazione IP55</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
@@ -6415,7 +6383,7 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce E.12 (2 scatole per 2 linee)</t>
+          <t>regola Nove C per le linee elettriche dedicate</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -6432,7 +6400,7 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>fluidi/power_supply/corrugato-di-potenza</t>
+          <t>Tubo corrugato Ø25 per le linee di alimentazione</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
@@ -6442,7 +6410,7 @@
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce E.10 (40 m per 35 m di linee); l'arrotondamento a 10 m è della sessione di sviluppo, che riproduce il kit: da confermare</t>
+          <t>stima Nove C (corrugato a decine di metri)</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -6459,7 +6427,7 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>fluidi/interconnection/cavo-di-collegamento</t>
+          <t>Cavo di collegamento 4G1,5 a doppio isolamento, Collegamento UI-UE</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
@@ -6469,7 +6437,7 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 (cavo a 4 conduttori ≥ 1,5 mm² a doppio isolamento, dal manuale di installazione Daikin FTXM60-71A citato in RAPPORTO.md §10)</t>
+          <t>manuale di installazione del costruttore della macchina</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -6486,7 +6454,7 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>fluidi/control_bus/cavo-di-bus</t>
+          <t>Cavo 2×0,75 (P1-P2), Linea P1-P2 dell'unita' interna</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
@@ -6496,7 +6464,7 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 (bus a stella dalla centrale; P1-P2 per gateway e comando a filo)</t>
+          <t>regola Nove C per i bus e le linee di comando</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -6513,7 +6481,7 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>fluidi/control_bus/cavo-di-bus</t>
+          <t>Cavo bus Airzone, schermato, Bus Airzone ai termostati</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
@@ -6523,7 +6491,7 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 (bus a stella dalla centrale; P1-P2 per gateway e comando a filo)</t>
+          <t>regola Nove C per i bus e le linee di comando</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -6540,7 +6508,7 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>fluidi/control_bus/corrugato-di-bus</t>
+          <t>Tubo corrugato Ø20 per bus e linee di comando</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
@@ -6550,7 +6518,7 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce E.11 (40 m per 37,5 m di bus); l'arrotondamento a 10 m è della sessione di sviluppo: da confermare</t>
+          <t>stima Nove C (corrugato a decine di metri)</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -6567,7 +6535,7 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>corredo/wired-remote/scatola-503 + corredo/room-thermostat/scatola-503</t>
+          <t>Scatola 503 per termostati e comandi a parete</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
@@ -6577,7 +6545,7 @@
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce E.13</t>
+          <t>regola Nove C per gli apparecchi a parete</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
@@ -6594,7 +6562,7 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>corredo/electrical-panel/aggiornamento-schema-quadro</t>
+          <t>Aggiornamento dello schema del quadro elettrico</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
@@ -6604,7 +6572,7 @@
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce E.6; REVISIONE-INDIPENDENTE.md rilievo 12</t>
+          <t>regola Nove C per le linee elettriche dedicate</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -6621,7 +6589,7 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>corredo/isolator-switch/sezionatore</t>
+          <t>Sezionatore onnipolare di prossimità IP55, apertura contatti ≥ 3 mm</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
@@ -6631,7 +6599,7 @@
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: RAPPORTO.md §7 (apertura dei contatti ≥ 3 mm dal manuale di installazione Daikin FTXM60-71A, citato in RAPPORTO.md §10)</t>
+          <t>manuale di installazione del costruttore della macchina (apertura dei contatti)</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
@@ -6648,7 +6616,7 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>fluidi/supply_air/foratura-per-flessibile</t>
+          <t>Foratura di tramezza Ø250 (o vano 450×250) per flessibili e plenum di bocchetta</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
@@ -6658,7 +6626,7 @@
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce F.3; REVISIONE-INDIPENDENTE.md rilievi 1 e 11 (le aperture sono dell'installatore)</t>
+          <t>regola Nove C per le assistenze murarie</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
@@ -6675,7 +6643,7 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>fluidi/refrigerant_gas/foratura-linee-frigo</t>
+          <t>Foratura di parete interna Ø80 per linee frigorifere e cavi</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
@@ -6685,7 +6653,7 @@
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce F.2; REVISIONE-INDIPENDENTE.md rilievo 11</t>
+          <t>regola Nove C per le assistenze murarie</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
@@ -6702,7 +6670,7 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>fluidi/condensate/foratura-condensa</t>
+          <t>Foratura per lo scarico della condensa</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
@@ -6712,7 +6680,7 @@
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce F.4</t>
+          <t>regola Nove C per le assistenze murarie</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
@@ -6729,7 +6697,7 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>corredo/wired-remote/traccia-per-apparecchio-a-parete + corredo/room-thermostat/traccia-per-apparecchio-a-parete</t>
+          <t>Traccia per termostati e comandi a parete</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
@@ -6739,7 +6707,7 @@
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce F.7</t>
+          <t>regola Nove C per gli apparecchi a parete</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
@@ -6756,7 +6724,7 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>corredo/electrical-panel/tracce-dal-quadro</t>
+          <t>Tracce per le linee dal quadro al controsoffitto</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
@@ -6766,7 +6734,7 @@
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce F.6 (5 m per due linee); 2,5 m di discesa per linea è della sessione di sviluppo, che riproduce il kit: da confermare</t>
+          <t>stima Nove C (2,5 m di traccia per linea)</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
@@ -6783,17 +6751,17 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>corredo/condensate-outlet/traccia-condensa</t>
+          <t>Traccia per la condensa fino allo scarico</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>scarico: 3</t>
+          <t>AL-01: 3</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce F.5 (3 m nel bagno)</t>
+          <t>stima Nove C (3 m di traccia fino allo scarico)</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
@@ -6810,7 +6778,7 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>corredo/split-outdoor-unit/carotaggio-parete-esterna</t>
+          <t>Carotaggio parete esterna Ø80 con guaina passante e sigillatura</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
@@ -6820,7 +6788,7 @@
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce F.1</t>
+          <t>regola Nove C per le assistenze murarie</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
@@ -6837,7 +6805,7 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>fluidi/supply_air/velette-per-le-bocchette</t>
+          <t>Velette o controsoffitti per le bocchette, altezza utile ≥ 30 cm</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
@@ -6847,7 +6815,7 @@
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce Z.3; REVISIONE-INDIPENDENTE.md rilievo 5</t>
+          <t>regola Nove C per le bocchette in controsoffitto</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
@@ -6864,7 +6832,7 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>corredo/air-supply-terminal/bocchetta-di-mandata</t>
+          <t>Bocchetta di mandata 400×200 a doppio filare con serranda</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
@@ -6874,12 +6842,12 @@
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce Z.4 (bocchette del committente nell'offerta del caso)</t>
+          <t>regola Nove C per le bocchette di mandata</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>Chi fornisce le bocchette lo dice l'offerta: nel kit sono del committente. Se le fornisce l'installatore, si cambia la fornitura di questa voce, qui: la distinta non legge la fornitura dal grafo.</t>
+          <t>Chi fornisce le bocchette è una scelta dell'offerta (`distinta.json`, fornitura «bocchette_e_griglie»): nelle offerte Nove C sono del Committente.</t>
         </is>
       </c>
     </row>
@@ -6891,22 +6859,22 @@
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>corredo/air-supply-terminal/griglia-di-transito</t>
+          <t>Griglia di transito o luce sotto porta per il ritorno dell'aria dal locale servito</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>5 pezzi × 1 = 5 (B1, B2, B3, B4, B5)</t>
+          <t>4: 4 locali serviti (Camera 13 m², Camera 15 m², Camera 16 m², Soggiorno-cucina); il locale e' letto dall'etichetta della bocchetta</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce Z.6; REVISIONE-INDIPENDENTE.md rilievo 28</t>
+          <t>regola Nove C per il ritorno dell'aria</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>Senza un passaggio, l'aria immessa non torna alla ripresa: la portata cala e cresce il rumore. L'area efficace minima per bocchetta è nella verifica dell'aria.</t>
+          <t>Senza un passaggio, l'aria immessa non torna alla ripresa: la portata cala e cresce il rumore. Una per locale servito, non per bocchetta: due bocchette nello stesso locale ne vogliono una sola, e un locale con un varco aperto verso la ripresa nessuna. Il locale è il dato `locale` della bocchetta (o, se manca, la sua etichetta senza le parentesi); il varco è `varco` sulla bocchetta. L'area efficace minima per locale è nella verifica dell'aria.</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6886,7 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>corredo/zoning-plenum-5/botola-di-ispezione + corredo/ducted-indoor-unit/botola-di-ispezione</t>
+          <t>Botola di ispezione ≥ 600×600 sotto la macchina (filtro, pompa, scheda)</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
@@ -6928,7 +6896,7 @@
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce Z.2 («sotto UI … e sotto plenum e centrale», n 2)</t>
+          <t>regola Nove C per la posa del plenum di zona; regola Nove C per la posa dell'unità interna canalizzata</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
@@ -6945,7 +6913,7 @@
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>corredo/return-air-terminal/griglia-di-ripresa</t>
+          <t>Griglia di ripresa 1000×250 senza filtro, apribile per accedere al filtro</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
@@ -6955,7 +6923,7 @@
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce Z.5</t>
+          <t>regola Nove C per la ripresa dell'aria</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
@@ -6972,7 +6940,7 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>corredo/ducted-indoor-unit/controsoffitto-zona-macchina</t>
+          <t>Controsoffitto in zona unità interna e plenum: altezza libera ≥ 35 cm sotto il solaio</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
@@ -6982,7 +6950,7 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce Z.1 (altezza della FBA60A9 245 mm più sospensioni e pendenza della condensa)</t>
+          <t>regola Nove C per la posa dell'unità interna canalizzata (ingombro della macchina)</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
@@ -6999,7 +6967,7 @@
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>attivita/chiusure-e-ripristini</t>
+          <t>Chiusura e ripristino di fori, tracce e passaggi</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
@@ -7009,7 +6977,7 @@
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, voce Z.7; REVISIONE-INDIPENDENTE.md rilievo 11 (l'offerta esclude chiusure e ripristini)</t>
+          <t>regola Nove C per le offerte a corpo (aperture all'installatore, chiusure a chi fa le opere edili)</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
@@ -7026,17 +6994,17 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>attivita/posa-unita-interna</t>
+          <t>Posa dell'unità interna in controsoffitto su sospensioni antivibranti, con plenum di zona e plenum di ripresa.</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: ducted-indoor-unit</t>
+          <t>nell'impianto: Unità interna canalizzata ad espansione diretta</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[0]</t>
+          <t>regola Nove C per le offerte a corpo</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
@@ -7053,17 +7021,17 @@
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>attivita/posa-unita-esterna</t>
+          <t>Posa dell'unità esterna su staffe con antivibranti; canalina esterna e scarico condensa dell'unità esterna.</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: split-outdoor-unit</t>
+          <t>nell'impianto: Unità esterna split a pompa di calore</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[1]</t>
+          <t>regola Nove C per le offerte a corpo</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
@@ -7080,17 +7048,17 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>attivita/linee-frigorifere-e-prove</t>
+          <t>Linee frigorifere: posa e cartelle; prova di tenuta in azoto prima della chiusura del controsoffitto, circuito lasciato in pressione con manometro fino al secondo accesso, con verbale; vuoto, apertura rubinetti, eventuale carica, registrazione F-Gas.</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: refrigerant_liquid, refrigerant_gas</t>
+          <t>nell'impianto: fluido frigorigeno in fase liquida, fluido frigorigeno in fase gassosa</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[2]; REVISIONE-INDIPENDENTE.md rilievo 14 (prove fra i due accessi)</t>
+          <t>regola Nove C per le prove delle linee frigorifere; regolamento F-Gas</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
@@ -7107,17 +7075,17 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>attivita/distribuzione-aria</t>
+          <t>Distribuzione aria: 5 rami flessibili con plenum porta-bocchetta, sostegni e sigillature; bocche protette fino alla posa delle bocchette.</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: supply_air</t>
+          <t>nell'impianto: aria di mandata</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[3]</t>
+          <t>regola Nove C per le offerte a corpo</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
@@ -7134,17 +7102,17 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>attivita/scarico-condensa-e-prova</t>
+          <t>Scarico condensa con sifone e allaccio allo scarico; prova di scarico e della pompa prima della chiusura del controsoffitto.</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: condensate</t>
+          <t>nell'impianto: condensa</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[4]; REVISIONE-INDIPENDENTE.md rilievo 14</t>
+          <t>regola Nove C per le offerte a corpo</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
@@ -7161,17 +7129,17 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>attivita/linee-elettriche-e-comandi</t>
+          <t>Linee elettriche dedicate dal quadro, collegamento fra le unità, linee di comando e bus; posa di termostati e comandi a parete.</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: power_supply, interconnection, control_bus</t>
+          <t>nell'impianto: alimentazione elettrica, collegamento elettrico fra le unita', bus di comando</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[5]</t>
+          <t>regola Nove C per le offerte a corpo</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
@@ -7188,17 +7156,17 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>attivita/messa-in-servizio</t>
+          <t>Messa in servizio con Nove C, al secondo accesso: regolazione della prevalenza dell'unità interna e misura delle portate per zona, configurazione della zonizzazione e dei comandi, app; collaudo con verbale.</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: ducted-indoor-unit, split-outdoor-unit</t>
+          <t>nell'impianto: Unità interna canalizzata ad espansione diretta, Unità esterna split a pompa di calore</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[6]; REVISIONE-INDIPENDENTE.md rilievi 8 e 16 (collaudo con portate misurate e verbale)</t>
+          <t>regola Nove C per le offerte a corpo</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
@@ -7215,17 +7183,17 @@
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>attivita/dico-elettrico</t>
+          <t>Dichiarazione di conformità D.M. 37/2008, art. 1 lettera a) (impianti elettrici), con lo schema del quadro aggiornato e gli allegati.</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: power_supply</t>
+          <t>nell'impianto: alimentazione elettrica</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[7]; REVISIONE-INDIPENDENTE.md rilievo 16 (due DiCo)</t>
+          <t>D.M. 37/2008</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
@@ -7242,17 +7210,17 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>attivita/dico-climatizzazione</t>
+          <t>Dichiarazione di conformità D.M. 37/2008, art. 1 lettera c) (impianti di climatizzazione), con allegati; documenti per libretto di impianto, catasto regionale e F-Gas.</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: refrigerant_liquid, refrigerant_gas, supply_air</t>
+          <t>nell'impianto: fluido frigorigeno in fase liquida, fluido frigorigeno in fase gassosa, aria di mandata</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[7]; REVISIONE-INDIPENDENTE.md rilievo 16</t>
+          <t>D.M. 37/2008</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
@@ -7269,7 +7237,7 @@
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>attivita/cantiere</t>
+          <t>Cantiere: POS e oneri della sicurezza (presenza dell'impresa del Committente), trabattello e mezzi di sollevamento.</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
@@ -7279,7 +7247,7 @@
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[8]; REVISIONE-INDIPENDENTE.md rilievo 13</t>
+          <t>regola Nove C per le offerte a corpo</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
@@ -7296,17 +7264,17 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>attivita/custodia-e-protezioni</t>
+          <t>Trasporto, ricevimento e custodia delle apparecchiature fornite da Nove C fino al collaudo; protezioni delle macchine e delle bocche durante le opere edili.</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: split-outdoor-unit, ducted-indoor-unit, zoning-plenum-5</t>
+          <t>nell'impianto: Unità esterna split a pompa di calore, Unità interna canalizzata ad espansione diretta, Plenum motorizzato di zona a cinque serrande</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[9]; REVISIONE-INDIPENDENTE.md rilievo 13</t>
+          <t>regola Nove C per le offerte a corpo</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
@@ -7323,7 +7291,7 @@
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>attivita/pulizia-e-smaltimenti</t>
+          <t>Pulizia finale e smaltimento di imballi e residui di lavorazione.</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
@@ -7333,7 +7301,7 @@
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, ATTIVITA[10]; REVISIONE-INDIPENDENTE.md rilievo 13</t>
+          <t>regola Nove C per le offerte a corpo</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
@@ -7350,17 +7318,17 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>attivita/variante-linea-frigorifera</t>
+          <t>Linea frigorifera completa oltre la quantità di computo (coppia pre-isolata, cavo di collegamento, canalina, refrigerante)</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: refrigerant_liquid, refrigerant_gas; solo prezzo unitario</t>
+          <t>nell'impianto: fluido frigorigeno in fase liquida, fluido frigorigeno in fase gassosa; solo prezzo unitario</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, VARIANTI V.1; REVISIONE-INDIPENDENTE.md rilievi 10 e 20</t>
+          <t>regola Nove C per le varianti a prezzo unitario</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
@@ -7377,17 +7345,17 @@
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>attivita/variante-flessibile</t>
+          <t>Flessibile posato oltre la quantità di computo, con fascette e sostegni</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: supply_air; solo prezzo unitario</t>
+          <t>nell'impianto: aria di mandata; solo prezzo unitario</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, VARIANTI V.2</t>
+          <t>regola Nove C per le varianti a prezzo unitario</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
@@ -7404,17 +7372,17 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>attivita/variante-cavo</t>
+          <t>Cavo di alimentazione in corrugato oltre la quantità di computo, stessa sezione</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: power_supply; solo prezzo unitario</t>
+          <t>nell'impianto: alimentazione elettrica; solo prezzo unitario</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, VARIANTI V.3</t>
+          <t>regola Nove C per le varianti a prezzo unitario</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
@@ -7431,7 +7399,7 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>attivita/variante-accesso</t>
+          <t>Accesso aggiuntivo in cantiere (oltre i due previsti)</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
@@ -7441,7 +7409,7 @@
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, VARIANTI V.4; REVISIONE-INDIPENDENTE.md rilievo 14 (terzo accesso)</t>
+          <t>regola Nove C per le varianti a prezzo unitario</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
@@ -7458,17 +7426,17 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>attivita/variante-centralino</t>
+          <t>Centralino aggiuntivo 8 moduli, se il quadro non ha i moduli liberi per le protezioni nuove</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>nel grafo: electrical-panel; solo prezzo unitario</t>
+          <t>nell'impianto: Quadro elettrico; solo prezzo unitario</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>kit AA-01: lavoro/dimensionamento.py, VARIANTI V.5; REVISIONE-INDIPENDENTE.md rilievo 12</t>
+          <t>regola Nove C per le varianti a prezzo unitario</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
@@ -7488,7 +7456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7498,7 +7466,7 @@
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>Note, domande al progettista e avvisi</t>
+          <t>Note, cose da confermare, domande al progettista e avvisi</t>
         </is>
       </c>
     </row>
@@ -7562,31 +7530,31 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>La distinta non progetta: lunghezze, sezioni, portate, protezioni, marca e modello sono dati del progettista; la distinta li maggiora e ne conta il corredo con regole scritte, ciascuna con la sua fonte (regole cfc42a99c0fd0a1a).</t>
+          <t>Fornitura da confermare: apparecchiature fornite da Nove C; bocchette e griglie, opere edili del Committente; messa in servizio con Nove C.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Avviso</t>
+          <t>Nota</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>T09 (Scarico condensa: UI-01 - sifone - scarico): c-2 senza lunghezza; si considera compresa nei 7,6 m dati sul tratto.</t>
+          <t>La distinta non progetta: lunghezze, sezioni, portate, protezioni, marca e modello sono dati del progettista; la distinta li maggiora e ne conta il corredo con regole scritte, ciascuna con la sua fonte (regole dea73506dac30790).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Avviso</t>
+          <t>Da confermare</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>T10 (Alimentazione unita' esterna: QE-01 - SZ-01 - UE-01): e-1a senza lunghezza; si considera compresa nei 15 m dati sul tratto.</t>
+          <t>Fornitura: apparecchiature fornite da Nove C; bocchette e griglie del Committente; opere edili del Committente; messa in servizio con Nove C — come da regole predefinite di Nove C; confermare per questa offerta.</t>
         </is>
       </c>
     </row>
@@ -7598,7 +7566,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>T02, T04, T05 (aria di mandata): attraversamenti di parete non dati, assunti 1 per tratto (kit AA-01: lavoro/dimensionamento.py, voce F «Foratura di tramezza … n 7: 5 bocchette e 2 nella tramezza fra i disimpegni»).</t>
+          <t>T09 (Scarico condensa: UI-01 - SIF-01 - AL-01): la tubazione SIF-01 - AL-01 senza lunghezza; si considera compresa nei 7,6 m dati sul tratto.</t>
         </is>
       </c>
     </row>
@@ -7610,7 +7578,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>T09 (condensa): attraversamenti di parete non dati, assunti 1 per tratto (kit AA-01: lavoro/dimensionamento.py, voce F.4 «Foratura per la condensa verso il bagno»).</t>
+          <t>T10 (Alimentazione unita' esterna: QE-01 - SZ-01 - UE-01): la tubazione SZ-01 - UE-01 senza lunghezza; si considera compresa nei 15 m dati sul tratto.</t>
         </is>
       </c>
     </row>
@@ -7621,6 +7589,30 @@
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>T02, T04, T05 (aria di mandata): attraversamenti di parete non dati, assunti 1 per tratto (regola Nove C: una parete per ramo, se il progettista non dice quante).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Avviso</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>T09 (condensa): attraversamenti di parete non dati, assunti 1 per tratto (regola Nove C: una parete, se il progettista non dice quante).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Avviso</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>T13, scritta sulla tavola: «P1-P2 · L 3 m», contro L 5 m da quotare.</t>
         </is>

</xml_diff>

<commit_message>
Uscite rifatte: AA-01 (REL-013), la M.02, il caso corretto del T1 e lo schema del T3
- docs/collaudi/REL-013/AA-01*: la distinta con la numerazione per sigle e il plenum
  di ripresa; il RAPPORTO dice, al §8, che cosa cambia rispetto al kit.
- docs/collaudi/REL-012/fase-2: la M.02 (rifai.sh), 0 bloccanti, con i quattro
  termostati Airzone Blueface nella tabella delle apparecchiature.
- docs/collaudi/REL-012/collaudo-t1/correzioni: rifatta col piano ricomposto
  (bocchette e termostati a x=225), 0 bloccanti.
- docs/collaudi/REL-012/collaudo-t3/rifatto: nuovo, lo schema e la distinta del
  collaudo T3 col grafo e il piano del collaudo, e la consegna in un comando.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/collaudi/REL-012/fase-2/distinta/distinta.xlsx
+++ b/docs/collaudi/REL-012/fase-2/distinta/distinta.xlsx
@@ -598,7 +598,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Committente: Committente (dati omessi). Indirizzo: Indirizzo omesso. Allegata alla tavola M.02, rev. 00 del 29.10.2026. Regole della distinta dea73506dac30790. Quantità indicative.</t>
+          <t>Committente: Committente (dati omessi). Indirizzo: Indirizzo omesso. Allegata alla tavola M.02, rev. 00 del 29.10.2026. Regole della distinta f8b849f909489495. Quantità indicative.</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Cavo FG16OR16 3G2,5, Alimentazione unita' esterna</t>
+          <t>Cavo FG16OR16 3G1,5, Alimentazione centrale Airzone</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="D48" s="8" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>T10 stimati 15 m</t>
+          <t>T10 stimati 12 m</t>
         </is>
       </c>
       <c r="G48" s="11" t="n"/>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Cavo FG16OR16 3G1,5, Alimentazione centrale Airzone</t>
+          <t>Cavo FG16OR16 3G2,5, Alimentazione unita' esterna</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="D49" s="8" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>T11 stimati 12 m</t>
+          <t>T11 stimati 15 m</t>
         </is>
       </c>
       <c r="G49" s="11" t="n"/>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Magnetotermico-differenziale 1P+N C16, Idn 30 mA, tipo A o F, 6 kA, linea dedicata: Alimentazione unita' esterna</t>
+          <t>Magnetotermico 1P+N C6, linea dedicata: Alimentazione centrale Airzone</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Magnetotermico 1P+N C6, linea dedicata: Alimentazione centrale Airzone</t>
+          <t>Magnetotermico-differenziale 1P+N C16, Idn 30 mA, tipo A o F, 6 kA, linea dedicata: Alimentazione unita' esterna</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Cavo 2×0,75 (P1-P2), Linea P1-P2 dell'unita' interna</t>
+          <t>Cavo bus Airzone, schermato, Bus Airzone ai termostati</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="D55" s="8" t="n">
-        <v>10.5</v>
+        <v>29</v>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>T13 stimati 1,5 m; T14 stimati 3,7 m</t>
+          <t>T13 stimati 6,5 m; T14 stimati 4,9 m; T15 stimati 5,2 m; T16 stimati 3,7 m</t>
         </is>
       </c>
       <c r="G55" s="11" t="n"/>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Cavo bus Airzone, schermato, Bus Airzone ai termostati</t>
+          <t>Cavo 2×0,75 (P1-P2), Linea P1-P2 dell'unita' interna</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="D56" s="8" t="n">
-        <v>29</v>
+        <v>10.5</v>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>T15 stimati 6,5 m; T16 stimati 4,9 m; T17 stimati 5,2 m; T18 stimati 3,7 m</t>
+          <t>T17 stimati 3,7 m; T18 stimati 1,5 m</t>
         </is>
       </c>
       <c r="G56" s="11" t="n"/>
@@ -3744,7 +3744,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>canale di ripresa coibentato</t>
+          <t>plenum di ripresa coibentato</t>
         </is>
       </c>
       <c r="F9" s="7" t="n">
@@ -3889,17 +3889,17 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Alimentazione unita' esterna</t>
+          <t>Alimentazione centrale Airzone</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>QE-01 - SZ-01 - UE-01</t>
+          <t>QE-01 - CZ-01</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>3G2,5</t>
+          <t>3G1,5</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -3910,14 +3910,14 @@
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="7" t="n"/>
       <c r="H13" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="I13" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="I13" s="7" t="n">
-        <v>20</v>
-      </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>(15 + 1) × 1,15 = 18,4 → 18,5 m; minimo scritto sul tratto 20 m → 20 m</t>
+          <t>(12 + 1) × 1,15 = 14,95 → 15 m</t>
         </is>
       </c>
     </row>
@@ -3929,17 +3929,17 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Alimentazione centrale Airzone</t>
+          <t>Alimentazione unita' esterna</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>QE-01 - CZ-01</t>
+          <t>QE-01 - SZ-01 - UE-01</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>3G1,5</t>
+          <t>3G2,5</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -3950,14 +3950,14 @@
       <c r="F14" s="7" t="n"/>
       <c r="G14" s="7" t="n"/>
       <c r="H14" s="7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>(12 + 1) × 1,15 = 14,95 → 15 m</t>
+          <t>(15 + 1) × 1,15 = 18,4 → 18,5 m; minimo scritto sul tratto 20 m → 20 m</t>
         </is>
       </c>
     </row>
@@ -4009,17 +4009,17 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Linea P1-P2 dell'unita' interna</t>
+          <t>Bus Airzone ai termostati</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>UI-01 - CZ-01</t>
+          <t>CZ-01 - TZ-01</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>2×0,75 (P1-P2)</t>
+          <t>bus Airzone, schermato</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -4030,14 +4030,14 @@
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="7" t="n"/>
       <c r="H16" s="7" t="n">
-        <v>1.5</v>
+        <v>6.5</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>(1,5 + 1) × 1,15 = 2,88 → 3 m; minimo bus 5 m → 5 m</t>
+          <t>(6,5 + 1) × 1,15 = 8,62 → 9 m</t>
         </is>
       </c>
     </row>
@@ -4049,17 +4049,17 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Linea P1-P2 dell'unita' interna</t>
+          <t>Bus Airzone ai termostati</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>UI-01 - CF-01</t>
+          <t>CZ-01 - TZ-02</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>2×0,75 (P1-P2)</t>
+          <t>bus Airzone, schermato</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -4070,14 +4070,14 @@
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7" t="n"/>
       <c r="H17" s="7" t="n">
-        <v>3.7</v>
+        <v>4.9</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>5.5</v>
+        <v>7</v>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>(3,7 + 1) × 1,15 = 5,4 → 5,5 m</t>
+          <t>(4,9 + 1) × 1,15 = 6,79 → 7 m</t>
         </is>
       </c>
     </row>
@@ -4094,7 +4094,7 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>CZ-01 - TZ-01</t>
+          <t>CZ-01 - TZ-03</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -4110,14 +4110,14 @@
       <c r="F18" s="7" t="n"/>
       <c r="G18" s="7" t="n"/>
       <c r="H18" s="7" t="n">
-        <v>6.5</v>
+        <v>5.2</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>(6,5 + 1) × 1,15 = 8,62 → 9 m</t>
+          <t>(5,2 + 1) × 1,15 = 7,13 → 7,5 m</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4134,7 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>CZ-01 - TZ-02</t>
+          <t>CZ-01 - TZ-04</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -4150,14 +4150,14 @@
       <c r="F19" s="7" t="n"/>
       <c r="G19" s="7" t="n"/>
       <c r="H19" s="7" t="n">
-        <v>4.9</v>
+        <v>3.7</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>(4,9 + 1) × 1,15 = 6,79 → 7 m</t>
+          <t>(3,7 + 1) × 1,15 = 5,4 → 5,5 m</t>
         </is>
       </c>
     </row>
@@ -4169,17 +4169,17 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Bus Airzone ai termostati</t>
+          <t>Linea P1-P2 dell'unita' interna</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>CZ-01 - TZ-03</t>
+          <t>UI-01 - CF-01</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>bus Airzone, schermato</t>
+          <t>2×0,75 (P1-P2)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -4190,14 +4190,14 @@
       <c r="F20" s="7" t="n"/>
       <c r="G20" s="7" t="n"/>
       <c r="H20" s="7" t="n">
-        <v>5.2</v>
+        <v>3.7</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>(5,2 + 1) × 1,15 = 7,13 → 7,5 m</t>
+          <t>(3,7 + 1) × 1,15 = 5,4 → 5,5 m</t>
         </is>
       </c>
     </row>
@@ -4209,17 +4209,17 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Bus Airzone ai termostati</t>
+          <t>Linea P1-P2 dell'unita' interna</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>CZ-01 - TZ-04</t>
+          <t>UI-01 - CZ-01</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>bus Airzone, schermato</t>
+          <t>2×0,75 (P1-P2)</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -4230,14 +4230,14 @@
       <c r="F21" s="7" t="n"/>
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="7" t="n">
-        <v>3.7</v>
+        <v>1.5</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>(3,7 + 1) × 1,15 = 5,4 → 5,5 m</t>
+          <t>(1,5 + 1) × 1,15 = 2,88 → 3 m; minimo bus 5 m → 5 m</t>
         </is>
       </c>
     </row>
@@ -4955,12 +4955,12 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>«3G2,5 · L 20 m»</t>
+          <t>«3G1,5 · L 15 m»</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>L 20 m da quotare</t>
+          <t>L 15 m da quotare</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -4987,12 +4987,12 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>«3G1,5 · L 15 m»</t>
+          <t>«3G2,5 · L 20 m»</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>L 15 m da quotare</t>
+          <t>L 20 m da quotare</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -5051,17 +5051,17 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>«P1-P2 · L 3 m»</t>
+          <t>«bus · L 9 m»</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>L 5 m da quotare</t>
+          <t>L 9 m da quotare</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>oltre</t>
+          <t>entro</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -5083,12 +5083,12 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>«P1-P2 · L 5,5 m»</t>
+          <t>«bus · L 7 m»</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>L 5,5 m da quotare</t>
+          <t>L 7 m da quotare</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
@@ -5115,12 +5115,12 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>«bus · L 9 m»</t>
+          <t>«bus · L 7,5 m»</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>L 9 m da quotare</t>
+          <t>L 7,5 m da quotare</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -5147,12 +5147,12 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>«bus · L 7 m»</t>
+          <t>«bus · L 5,5 m»</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>L 7 m da quotare</t>
+          <t>L 5,5 m da quotare</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -5179,12 +5179,12 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>«bus · L 7,5 m»</t>
+          <t>«P1-P2 · L 5,5 m»</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>L 7,5 m da quotare</t>
+          <t>L 5,5 m da quotare</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -5211,17 +5211,17 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>«bus · L 5,5 m»</t>
+          <t>«P1-P2 · L 3 m»</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>L 5,5 m da quotare</t>
+          <t>L 5 m da quotare</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>entro</t>
+          <t>oltre</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
@@ -6265,12 +6265,12 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Cavo FG16OR16 3G2,5, Alimentazione unita' esterna</t>
+          <t>Cavo FG16OR16 3G1,5, Alimentazione centrale Airzone</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>T10 20 m</t>
+          <t>T10 15 m</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
@@ -6292,12 +6292,12 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Cavo FG16OR16 3G1,5, Alimentazione centrale Airzone</t>
+          <t>Cavo FG16OR16 3G2,5, Alimentazione unita' esterna</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>T11 15 m</t>
+          <t>T11 20 m</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
@@ -6319,7 +6319,7 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Magnetotermico-differenziale 1P+N C16, Idn 30 mA, tipo A o F, 6 kA, linea dedicata: Alimentazione unita' esterna</t>
+          <t>Magnetotermico 1P+N C6, linea dedicata: Alimentazione centrale Airzone</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Magnetotermico 1P+N C6, linea dedicata: Alimentazione centrale Airzone</t>
+          <t>Magnetotermico-differenziale 1P+N C16, Idn 30 mA, tipo A o F, 6 kA, linea dedicata: Alimentazione unita' esterna</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>T10 20 + T11 15 = 35 m × 1, per eccesso a 10 m = 40 m</t>
+          <t>T10 15 + T11 20 = 35 m × 1, per eccesso a 10 m = 40 m</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -6454,12 +6454,12 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Cavo 2×0,75 (P1-P2), Linea P1-P2 dell'unita' interna</t>
+          <t>Cavo bus Airzone, schermato, Bus Airzone ai termostati</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>T13 5 + T14 5,5 = 10,5 m</t>
+          <t>T13 9 + T14 7 + T15 7,5 + T16 5,5 = 29 m</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -6481,12 +6481,12 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Cavo bus Airzone, schermato, Bus Airzone ai termostati</t>
+          <t>Cavo 2×0,75 (P1-P2), Linea P1-P2 dell'unita' interna</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>T15 9 + T16 7 + T17 7,5 + T18 5,5 = 29 m</t>
+          <t>T17 5,5 + T18 5 = 10,5 m</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -6513,7 +6513,7 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>T13 5 + T14 5,5 + T15 9 + T16 7 + T17 7,5 + T18 5,5 = 39,5 m × 1, per eccesso a 10 m = 40 m</t>
+          <t>T13 9 + T14 7 + T15 7,5 + T16 5,5 + T17 5,5 + T18 5 = 39,5 m × 1, per eccesso a 10 m = 40 m</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>La distinta non progetta: lunghezze, sezioni, portate, protezioni, marca e modello sono dati del progettista; la distinta li maggiora e ne conta il corredo con regole scritte, ciascuna con la sua fonte (regole dea73506dac30790).</t>
+          <t>La distinta non progetta: lunghezze, sezioni, portate, protezioni, marca e modello sono dati del progettista; la distinta li maggiora e ne conta il corredo con regole scritte, ciascuna con la sua fonte (regole f8b849f909489495).</t>
         </is>
       </c>
     </row>
@@ -7578,7 +7578,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>T10 (Alimentazione unita' esterna: QE-01 - SZ-01 - UE-01): la tubazione SZ-01 - UE-01 senza lunghezza; si considera compresa nei 15 m dati sul tratto.</t>
+          <t>T11 (Alimentazione unita' esterna: QE-01 - SZ-01 - UE-01): la tubazione SZ-01 - UE-01 senza lunghezza; si considera compresa nei 15 m dati sul tratto.</t>
         </is>
       </c>
     </row>
@@ -7614,7 +7614,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>T13, scritta sulla tavola: «P1-P2 · L 3 m», contro L 5 m da quotare.</t>
+          <t>T18, scritta sulla tavola: «P1-P2 · L 3 m», contro L 5 m da quotare.</t>
         </is>
       </c>
     </row>

</xml_diff>